<commit_message>
Moves data centers into the buildings sector as a fourth building type; adds high/medium/low distributed capacity pathways for data centers; adds SYSHECF values explicitly for gas and petroleum distributed resources; addresses cash flow misalignment with data centers
</commit_message>
<xml_diff>
--- a/InputData/bldgs/BFoCSbQL/BAU Frac of Components Sold by Quality Lvl.xlsx
+++ b/InputData/bldgs/BFoCSbQL/BAU Frac of Components Sold by Quality Lvl.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Meghan\Dropbox (Energy Innovation)\EPS Versions\eps-1.5.0-us-wipI\InputData\bldgs\BFoCSbQL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\EPS Structure Research\eps-us-dc-replay\InputData\bldgs\BFoCSbQL\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5520360-7D46-4600-AF80-5E9C4C6C8D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="105" windowWidth="20115" windowHeight="9780"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -17,13 +18,27 @@
     <sheet name="BFoCSbQL-urban-residential" sheetId="3" r:id="rId3"/>
     <sheet name="BFoCSbQL-rural-residential" sheetId="5" r:id="rId4"/>
     <sheet name="BFoCSbQL-commercial" sheetId="4" r:id="rId5"/>
+    <sheet name="BFoCSbQL-data-centers" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="83">
   <si>
     <t>Source:</t>
   </si>
@@ -266,12 +281,18 @@
   </si>
   <si>
     <t>for energy efficient rebates.</t>
+  </si>
+  <si>
+    <t>Data centers</t>
+  </si>
+  <si>
+    <t>Data centers are a separate building type. Their export tab copies the commercial quality-level shares.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
@@ -350,7 +371,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -371,16 +392,14 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -400,9 +419,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -440,9 +459,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -477,7 +496,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -512,7 +531,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -685,8 +704,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -727,12 +746,12 @@
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
+      <c r="A9" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
+      <c r="A10" t="s">
         <v>80</v>
       </c>
     </row>
@@ -754,6 +773,14 @@
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -763,7 +790,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -893,40 +920,39 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+      <c r="A12" t="s">
         <v>65</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="2">
         <v>3519000</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="2">
         <v>0.27</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="E12" t="s">
         <v>11</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="12" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12" t="s">
+      <c r="B13" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="13">
+      <c r="C13" s="2">
         <v>1652000</v>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="2">
         <v>0.46</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="E13" t="s">
         <v>11</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="12" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1384,33 +1410,33 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F12" r:id="rId1"/>
-    <hyperlink ref="F8" r:id="rId2"/>
-    <hyperlink ref="F13" r:id="rId3"/>
-    <hyperlink ref="F14" r:id="rId4"/>
-    <hyperlink ref="F9" r:id="rId5"/>
-    <hyperlink ref="F10" r:id="rId6"/>
-    <hyperlink ref="F11" r:id="rId7"/>
-    <hyperlink ref="F15" r:id="rId8"/>
-    <hyperlink ref="F16" r:id="rId9"/>
-    <hyperlink ref="F17:F18" r:id="rId10" display="http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.8.xlsx"/>
-    <hyperlink ref="F19" r:id="rId11"/>
-    <hyperlink ref="F27" r:id="rId12"/>
-    <hyperlink ref="F28:F31" r:id="rId13" display="http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.13.xlsx"/>
-    <hyperlink ref="F20" r:id="rId14"/>
-    <hyperlink ref="F21" r:id="rId15"/>
-    <hyperlink ref="F25" r:id="rId16"/>
-    <hyperlink ref="F26" r:id="rId17"/>
-    <hyperlink ref="F22" r:id="rId18"/>
-    <hyperlink ref="F23" r:id="rId19"/>
-    <hyperlink ref="F24" r:id="rId20"/>
+    <hyperlink ref="F12" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="F8" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="F13" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="F14" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="F9" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
+    <hyperlink ref="F10" r:id="rId6" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
+    <hyperlink ref="F11" r:id="rId7" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
+    <hyperlink ref="F15" r:id="rId8" xr:uid="{00000000-0004-0000-0100-000007000000}"/>
+    <hyperlink ref="F16" r:id="rId9" xr:uid="{00000000-0004-0000-0100-000008000000}"/>
+    <hyperlink ref="F17:F18" r:id="rId10" display="http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.8.xlsx" xr:uid="{00000000-0004-0000-0100-000009000000}"/>
+    <hyperlink ref="F19" r:id="rId11" xr:uid="{00000000-0004-0000-0100-00000A000000}"/>
+    <hyperlink ref="F27" r:id="rId12" xr:uid="{00000000-0004-0000-0100-00000B000000}"/>
+    <hyperlink ref="F28:F31" r:id="rId13" display="http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.13.xlsx" xr:uid="{00000000-0004-0000-0100-00000C000000}"/>
+    <hyperlink ref="F20" r:id="rId14" xr:uid="{00000000-0004-0000-0100-00000D000000}"/>
+    <hyperlink ref="F21" r:id="rId15" xr:uid="{00000000-0004-0000-0100-00000E000000}"/>
+    <hyperlink ref="F25" r:id="rId16" xr:uid="{00000000-0004-0000-0100-00000F000000}"/>
+    <hyperlink ref="F26" r:id="rId17" xr:uid="{00000000-0004-0000-0100-000010000000}"/>
+    <hyperlink ref="F22" r:id="rId18" xr:uid="{00000000-0004-0000-0100-000011000000}"/>
+    <hyperlink ref="F23" r:id="rId19" xr:uid="{00000000-0004-0000-0100-000012000000}"/>
+    <hyperlink ref="F24" r:id="rId20" xr:uid="{00000000-0004-0000-0100-000013000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
@@ -1423,7 +1449,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="14" t="s">
         <v>78</v>
       </c>
       <c r="B1" s="10" t="s">
@@ -1463,11 +1489,11 @@
       <c r="A4" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="13">
         <f t="shared" si="0"/>
         <v>0.56609034267912772</v>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="13">
         <f>AVERAGE(C2:C3)</f>
         <v>0.43390965732087228</v>
       </c>
@@ -1521,7 +1547,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
@@ -1534,7 +1560,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="14" t="s">
         <v>78</v>
       </c>
       <c r="B1" s="10" t="s">
@@ -1574,11 +1600,11 @@
       <c r="A4" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="13">
         <f t="shared" si="0"/>
         <v>0.56609034267912772</v>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="13">
         <f>AVERAGE(C2:C3)</f>
         <v>0.43390965732087228</v>
       </c>
@@ -1629,7 +1655,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
@@ -1642,7 +1668,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="14" t="s">
         <v>78</v>
       </c>
       <c r="B1" s="10" t="s">
@@ -1682,11 +1708,11 @@
       <c r="A4" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="13">
         <f t="shared" si="0"/>
         <v>0.56609034267912772</v>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="13">
         <f>AVERAGE(C2:C3)</f>
         <v>0.43390965732087228</v>
       </c>
@@ -1737,4 +1763,106 @@
     <ignoredError sqref="C2:C3 C5:C7" formulaRange="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0EAAE55-897F-428C-8AEA-71687D9B2A94}">
+  <sheetPr>
+    <tabColor rgb="FF1F3864"/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2">
+        <f>'BFoCSbQL-commercial'!B2</f>
+        <v>0.40218068535825546</v>
+      </c>
+      <c r="C2">
+        <f>'BFoCSbQL-commercial'!C2</f>
+        <v>0.59781931464174454</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3">
+        <f>'BFoCSbQL-commercial'!B3</f>
+        <v>0.73</v>
+      </c>
+      <c r="C3">
+        <f>'BFoCSbQL-commercial'!C3</f>
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4">
+        <f>'BFoCSbQL-commercial'!B4</f>
+        <v>0.56609034267912772</v>
+      </c>
+      <c r="C4">
+        <f>'BFoCSbQL-commercial'!C4</f>
+        <v>0.43390965732087228</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5">
+        <f>'BFoCSbQL-commercial'!B5</f>
+        <v>0.8</v>
+      </c>
+      <c r="C5">
+        <f>'BFoCSbQL-commercial'!C5</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6">
+        <f>'BFoCSbQL-commercial'!B6</f>
+        <v>0.53711053089643168</v>
+      </c>
+      <c r="C6">
+        <f>'BFoCSbQL-commercial'!C6</f>
+        <v>0.46288946910356832</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7">
+        <f>'BFoCSbQL-commercial'!B7</f>
+        <v>0.30697620874904064</v>
+      </c>
+      <c r="C7">
+        <f>'BFoCSbQL-commercial'!C7</f>
+        <v>0.69302379125095936</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>